<commit_message>
update phase 3 + testcase phase 9
</commit_message>
<xml_diff>
--- a/Extra/TCPIP_TestCases.xlsx
+++ b/Extra/TCPIP_TestCases.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project_LTM\Extra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{390AB970-98EF-4329-BB81-DF706608AD9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5A6C1B6-ED45-4881-9C88-272BAB6E0F41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TestCases" sheetId="1" r:id="rId1"/>
-    <sheet name="Screenshots" sheetId="2" r:id="rId2"/>
+    <sheet name="Hình TC21 - Kiểm tra CPU khi ch" sheetId="8" r:id="rId2"/>
+    <sheet name="Hình TC22 - Kiểm tra RAM khi ch" sheetId="7" r:id="rId3"/>
+    <sheet name="Hình TC20 - Connect 10 Clients" sheetId="6" r:id="rId4"/>
+    <sheet name="Hình TC19 - Connect 5 Clients" sheetId="5" r:id="rId5"/>
+    <sheet name="Hình TC18 - Đồng bộ message" sheetId="4" r:id="rId6"/>
+    <sheet name="Hình TC17 - Đồng bộ trạng thái " sheetId="3" r:id="rId7"/>
+    <sheet name="Screenshots" sheetId="2" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="Hình_TC01____Khởi_động_Server">Screenshots!$A$2</definedName>
@@ -32,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="133">
   <si>
     <t>No</t>
   </si>
@@ -313,9 +319,6 @@
     <t>Trạng thái Room được đồng bộ chính xác</t>
   </si>
   <si>
-    <t>Hình TC01 - Start Server</t>
-  </si>
-  <si>
     <t>Hình TC01 -  Khởi động Server</t>
   </si>
   <si>
@@ -373,32 +376,92 @@
     <t>Hình TC17 - Đồng bộ trạng thái Room</t>
   </si>
   <si>
-    <t>IHình TC03 - Đăng ký tài khoản người dùng</t>
+    <t>Hình TC03 - Đăng ký tài khoản người dùng</t>
+  </si>
+  <si>
+    <t>Kiểm tra đồng bộ message</t>
+  </si>
+  <si>
+    <t>Gửi nhiều tin nhắn trong Room</t>
+  </si>
+  <si>
+    <t>Hình TC18 - Đồng bộ message</t>
+  </si>
+  <si>
+    <t>Kiểm tra nhiều user connect với server</t>
+  </si>
+  <si>
+    <t>Kết nối 5 clients vào server</t>
+  </si>
+  <si>
+    <t>Kết nối 10 clients vào server</t>
+  </si>
+  <si>
+    <t>Hình TC19 - Connect 5 Clients</t>
+  </si>
+  <si>
+    <t>Hình TC20 - Connect 10 Clients</t>
+  </si>
+  <si>
+    <t>Hình TC17 - Đồng bộ trạng thái</t>
+  </si>
+  <si>
+    <t>Kiểm tra CPU khi chạy nhiều clients</t>
+  </si>
+  <si>
+    <t>Kiểm tra Ram khi chạy nhiều clients</t>
+  </si>
+  <si>
+    <t>Sau khi connect 10 clients vào server</t>
+  </si>
+  <si>
+    <t>Trước khi connect 10 clients vào server</t>
+  </si>
+  <si>
+    <t>Hình TC22 - Kiểm tra RAM khi chạy nhiều clients</t>
+  </si>
+  <si>
+    <t>Hình TC21 - Kiểm tra CPU khi chạy nhiều clients</t>
+  </si>
+  <si>
+    <t>5 client kết nối đồng thời, chat bình thường</t>
+  </si>
+  <si>
+    <t>10 client kết nối đồng thời, chat bình thường</t>
+  </si>
+  <si>
+    <t>Server không crash, không mất message</t>
+  </si>
+  <si>
+    <t>CPU không vượt ngưỡng bất thường ~15%</t>
+  </si>
+  <si>
+    <t>RAM không tăng liên tục</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="13"/>
-      <name val="Times New Roman"/>
+      <name val="Cambria"/>
       <family val="1"/>
       <scheme val="major"/>
     </font>
     <font>
       <sz val="13"/>
       <color theme="1"/>
-      <name val="Times New Roman"/>
+      <name val="Cambria"/>
       <family val="1"/>
       <scheme val="major"/>
     </font>
@@ -406,7 +469,7 @@
       <b/>
       <sz val="13"/>
       <color theme="1"/>
-      <name val="Times New Roman"/>
+      <name val="Cambria"/>
       <family val="1"/>
       <scheme val="major"/>
     </font>
@@ -414,7 +477,30 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -455,7 +541,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -464,13 +550,30 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -490,6 +593,368 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>594361</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>571501</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>96923</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3A74607F-9982-E522-1575-ED76F31881FC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1203961" y="266700"/>
+          <a:ext cx="9121140" cy="3670703"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>434774</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>129629</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{721364B5-0AEC-E4C5-71C0-B8A8DC03CF86}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2133600" y="563880"/>
+          <a:ext cx="5006774" cy="1028789"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>549216</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>84243</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A63AB8BF-F1A5-7A75-8E61-046E39F9542F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1828800" y="2148840"/>
+          <a:ext cx="6645216" cy="4884843"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>190501</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>373381</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>32526</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FBBA2465-56E8-7DD7-2A68-BE6B7D1FBA6C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1409701" y="198120"/>
+          <a:ext cx="9326880" cy="5137926"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>167640</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>373380</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>154948</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{420FB924-F67C-1AB5-4A93-DB1FC2DE43D8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2606040" y="213360"/>
+          <a:ext cx="8740140" cy="4003048"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>586740</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>183373</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>107083</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BE6DDCAF-1DC9-F41B-EE4C-A597F05A5E76}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2415540" y="213360"/>
+          <a:ext cx="5692633" cy="4648603"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>541020</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>38101</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>143815</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>160021</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{12BF4E30-7077-DF79-71C6-BBE8199E050F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1150620" y="259081"/>
+          <a:ext cx="9965995" cy="4511040"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1175,21 +1640,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I18"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I23"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.09765625" customWidth="1"/>
+    <col min="1" max="1" width="14.109375" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="65.5" customWidth="1"/>
-    <col min="4" max="4" width="41.296875" customWidth="1"/>
-    <col min="5" max="5" width="58.59765625" customWidth="1"/>
-    <col min="6" max="6" width="16.59765625" customWidth="1"/>
-    <col min="7" max="7" width="16.09765625" customWidth="1"/>
-    <col min="8" max="8" width="16.69921875" customWidth="1"/>
-    <col min="9" max="9" width="43.8984375" customWidth="1"/>
+    <col min="3" max="3" width="65.44140625" customWidth="1"/>
+    <col min="4" max="4" width="41.33203125" customWidth="1"/>
+    <col min="5" max="5" width="58.5546875" customWidth="1"/>
+    <col min="6" max="6" width="16.5546875" customWidth="1"/>
+    <col min="7" max="7" width="16.109375" customWidth="1"/>
+    <col min="8" max="8" width="16.6640625" customWidth="1"/>
+    <col min="9" max="9" width="43.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="16.8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1229,7 +1694,7 @@
         <v>11</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>12</v>
@@ -1239,8 +1704,8 @@
       </c>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
-      <c r="I2" s="6" t="s">
-        <v>95</v>
+      <c r="I2" s="4" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
@@ -1254,7 +1719,7 @@
         <v>16</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>17</v>
@@ -1264,8 +1729,8 @@
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
-      <c r="I3" s="6" t="s">
-        <v>96</v>
+      <c r="I3" s="4" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
@@ -1290,7 +1755,7 @@
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
       <c r="I4" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
@@ -1314,8 +1779,8 @@
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
-      <c r="I5" s="6" t="s">
-        <v>99</v>
+      <c r="I5" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
@@ -1339,8 +1804,8 @@
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
-      <c r="I6" s="6" t="s">
-        <v>100</v>
+      <c r="I6" s="4" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
@@ -1364,8 +1829,8 @@
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
-      <c r="I7" s="6" t="s">
-        <v>101</v>
+      <c r="I7" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
@@ -1389,8 +1854,8 @@
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
-      <c r="I8" s="6" t="s">
-        <v>102</v>
+      <c r="I8" s="4" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
@@ -1415,7 +1880,7 @@
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
@@ -1439,8 +1904,8 @@
       </c>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
-      <c r="I10" s="6" t="s">
-        <v>104</v>
+      <c r="I10" s="4" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
@@ -1464,8 +1929,8 @@
       </c>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
-      <c r="I11" s="6" t="s">
-        <v>105</v>
+      <c r="I11" s="4" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
@@ -1490,7 +1955,7 @@
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
@@ -1515,7 +1980,7 @@
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
@@ -1540,7 +2005,7 @@
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
@@ -1565,7 +2030,7 @@
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
@@ -1590,7 +2055,7 @@
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
@@ -1615,7 +2080,7 @@
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
@@ -1635,12 +2100,107 @@
         <v>92</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
-      <c r="I18" s="1" t="s">
-        <v>112</v>
+      <c r="I18" s="11" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="C19" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+      <c r="I19" s="15" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="C20" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="E20" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="11" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="C21" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="14"/>
+      <c r="H21" s="14"/>
+      <c r="I21" s="11" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="C22" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14"/>
+      <c r="I22" s="11" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="C23" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="14"/>
+      <c r="H23" s="14"/>
+      <c r="I23" s="16" t="s">
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -1653,29 +2213,260 @@
     <hyperlink ref="I8" location="Hình_TC07___Tham_gia_phòng_Chat" display="Hình TC07 - Tham gia phòng Chat" xr:uid="{828B66B9-6FBA-4E46-BD46-A6336762C3DF}"/>
     <hyperlink ref="I10" location="Hình_TC09___Tạo_phòng_Chat_mới" display="Hình TC09 - Tạo phòng Chat mới" xr:uid="{F889D5A5-A32E-40FD-B40A-52505BE28EC3}"/>
     <hyperlink ref="I11" location="Hình_TC10___Trao_đổi_tin_nhắn_trong_Room" display="Hình TC10 - Trao đổi tin nhắn trong Room" xr:uid="{2AE2DB4D-F54B-4FEB-8FD8-89877BE2D7CB}"/>
+    <hyperlink ref="I19" location="'Hình TC18 - Đồng bộ message'!A1" display="Hình TC18 - Đồng bộ message" xr:uid="{C3AA513E-00B7-4B29-8EF0-539D06E92FB2}"/>
+    <hyperlink ref="I18" location="'Hình TC17 - Đồng bộ trạng thái '!A1" display="Hình TC17 - Đồng bộ trạng thái" xr:uid="{D74CD5E5-1739-4F87-8BBD-E77D3BDA25B5}"/>
+    <hyperlink ref="I20" location="'Hình TC19 - Connect 5 Clients'!A1" display="Hình TC19 - Connect 5 Clients" xr:uid="{2195BCA0-0E0A-4590-980F-CE77378B883A}"/>
+    <hyperlink ref="I21" location="'Hình TC20 - Connect 10 Clients'!A1" display="Hình TC20 - Connect 10 Clients" xr:uid="{1CCAC8E6-01DC-4B4D-B74D-9FE8862BD535}"/>
+    <hyperlink ref="I23" location="'Hình TC22 - Kiểm tra RAM khi ch'!A1" display="'Hình TC22 - Kiểm tra RAM khi chạy nhiều clients" xr:uid="{1F374F00-DCE1-469A-AD42-95676046D49B}"/>
+    <hyperlink ref="I22" location="'Hình TC21 - Kiểm tra CPU khi ch'!A1" display="'Hình TC21 - Kiểm tra CPU khi chạy nhiều clients" xr:uid="{A01A1B81-F186-4FF7-B35C-786C9F6DA579}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{972460E1-2410-4833-9BFB-5E11EB484CF4}">
+  <dimension ref="C1:Q1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="3:17" x14ac:dyDescent="0.3">
+      <c r="C1" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C1:Q1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7E79FD0-FCD7-4E12-B613-849CA637A0C0}">
+  <dimension ref="E1:M11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E1" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+    </row>
+    <row r="3" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E3" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+    </row>
+    <row r="4" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
+    </row>
+    <row r="11" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E11" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
+      <c r="L11" s="6"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="E11:L11"/>
+    <mergeCell ref="E3:L3"/>
+    <mergeCell ref="E1:M1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{602CD738-ADA1-4281-82B2-C3922F24F61A}">
+  <dimension ref="D1:R1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="4:18" x14ac:dyDescent="0.3">
+      <c r="D1" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="D1:R1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33A06020-F75E-4644-8F10-0797C4350C85}">
+  <dimension ref="F1:S2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="6:19" x14ac:dyDescent="0.3">
+      <c r="F1" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
+      <c r="S1" s="6"/>
+    </row>
+    <row r="2" spans="6:19" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="G2" s="10"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="F1:S1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6207281B-3425-4D6E-A0BE-1A1B9E70A2FF}">
+  <dimension ref="E1:N1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="5:14" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="E1" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+      <c r="N1" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDC0F71C-E3BE-4001-B400-B8E200596A11}">
+  <dimension ref="C1:Q1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="3:17" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="C1" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C1:Q1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F3BF068-20E5-4563-9A01-7F8D1605D19B}">
   <dimension ref="A2:Y257"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="1:25" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
+        <v>93</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
       <c r="L2" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="5"/>
@@ -1693,128 +2484,128 @@
     </row>
     <row r="44" spans="1:17" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="B44" s="4"/>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
-      <c r="E44" s="4"/>
-      <c r="F44" s="4"/>
-      <c r="G44" s="4"/>
-      <c r="H44" s="4"/>
-      <c r="I44" s="4"/>
-      <c r="J44" s="4"/>
-      <c r="K44" s="4"/>
-      <c r="L44" s="4"/>
-      <c r="M44" s="4"/>
-      <c r="N44" s="4"/>
-      <c r="O44" s="4"/>
-      <c r="P44" s="4"/>
-      <c r="Q44" s="4"/>
+        <v>98</v>
+      </c>
+      <c r="B44" s="6"/>
+      <c r="C44" s="6"/>
+      <c r="D44" s="6"/>
+      <c r="E44" s="6"/>
+      <c r="F44" s="6"/>
+      <c r="G44" s="6"/>
+      <c r="H44" s="6"/>
+      <c r="I44" s="6"/>
+      <c r="J44" s="6"/>
+      <c r="K44" s="6"/>
+      <c r="L44" s="6"/>
+      <c r="M44" s="6"/>
+      <c r="N44" s="6"/>
+      <c r="O44" s="6"/>
+      <c r="P44" s="6"/>
+      <c r="Q44" s="6"/>
     </row>
     <row r="89" spans="2:16" ht="16.8" x14ac:dyDescent="0.3">
       <c r="B89" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="C89" s="4"/>
-      <c r="D89" s="4"/>
-      <c r="E89" s="4"/>
-      <c r="F89" s="4"/>
-      <c r="G89" s="4"/>
-      <c r="H89" s="4"/>
-      <c r="I89" s="4"/>
-      <c r="J89" s="4"/>
-      <c r="K89" s="4"/>
-      <c r="L89" s="4"/>
-      <c r="M89" s="4"/>
-      <c r="N89" s="4"/>
-      <c r="O89" s="4"/>
-      <c r="P89" s="4"/>
+        <v>99</v>
+      </c>
+      <c r="C89" s="6"/>
+      <c r="D89" s="6"/>
+      <c r="E89" s="6"/>
+      <c r="F89" s="6"/>
+      <c r="G89" s="6"/>
+      <c r="H89" s="6"/>
+      <c r="I89" s="6"/>
+      <c r="J89" s="6"/>
+      <c r="K89" s="6"/>
+      <c r="L89" s="6"/>
+      <c r="M89" s="6"/>
+      <c r="N89" s="6"/>
+      <c r="O89" s="6"/>
+      <c r="P89" s="6"/>
     </row>
     <row r="125" spans="2:16" ht="16.8" x14ac:dyDescent="0.3">
       <c r="B125" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="C125" s="4"/>
-      <c r="D125" s="4"/>
-      <c r="E125" s="4"/>
-      <c r="F125" s="4"/>
-      <c r="G125" s="4"/>
-      <c r="H125" s="4"/>
-      <c r="I125" s="4"/>
-      <c r="J125" s="4"/>
-      <c r="K125" s="4"/>
-      <c r="L125" s="4"/>
-      <c r="M125" s="4"/>
-      <c r="N125" s="4"/>
-      <c r="O125" s="4"/>
-      <c r="P125" s="4"/>
+        <v>100</v>
+      </c>
+      <c r="C125" s="6"/>
+      <c r="D125" s="6"/>
+      <c r="E125" s="6"/>
+      <c r="F125" s="6"/>
+      <c r="G125" s="6"/>
+      <c r="H125" s="6"/>
+      <c r="I125" s="6"/>
+      <c r="J125" s="6"/>
+      <c r="K125" s="6"/>
+      <c r="L125" s="6"/>
+      <c r="M125" s="6"/>
+      <c r="N125" s="6"/>
+      <c r="O125" s="6"/>
+      <c r="P125" s="6"/>
     </row>
     <row r="175" spans="2:16" ht="16.8" x14ac:dyDescent="0.3">
       <c r="B175" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="C175" s="4"/>
-      <c r="D175" s="4"/>
-      <c r="E175" s="4"/>
-      <c r="F175" s="4"/>
-      <c r="G175" s="4"/>
-      <c r="H175" s="4"/>
-      <c r="I175" s="4"/>
-      <c r="J175" s="4"/>
-      <c r="K175" s="4"/>
-      <c r="L175" s="4"/>
-      <c r="M175" s="4"/>
-      <c r="N175" s="4"/>
-      <c r="O175" s="4"/>
-      <c r="P175" s="4"/>
+        <v>101</v>
+      </c>
+      <c r="C175" s="6"/>
+      <c r="D175" s="6"/>
+      <c r="E175" s="6"/>
+      <c r="F175" s="6"/>
+      <c r="G175" s="6"/>
+      <c r="H175" s="6"/>
+      <c r="I175" s="6"/>
+      <c r="J175" s="6"/>
+      <c r="K175" s="6"/>
+      <c r="L175" s="6"/>
+      <c r="M175" s="6"/>
+      <c r="N175" s="6"/>
+      <c r="O175" s="6"/>
+      <c r="P175" s="6"/>
     </row>
     <row r="221" spans="2:24" ht="16.8" x14ac:dyDescent="0.3">
       <c r="B221" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="C221" s="4"/>
-      <c r="D221" s="4"/>
-      <c r="E221" s="4"/>
-      <c r="F221" s="4"/>
-      <c r="G221" s="4"/>
-      <c r="H221" s="4"/>
-      <c r="I221" s="4"/>
-      <c r="J221" s="4"/>
-      <c r="K221" s="4"/>
-      <c r="L221" s="4"/>
-      <c r="M221" s="4"/>
-      <c r="N221" s="4"/>
-      <c r="O221" s="4"/>
-      <c r="P221" s="4"/>
-      <c r="Q221" s="4"/>
-      <c r="R221" s="4"/>
-      <c r="S221" s="4"/>
-      <c r="T221" s="4"/>
-      <c r="U221" s="4"/>
-      <c r="V221" s="4"/>
-      <c r="W221" s="4"/>
-      <c r="X221" s="4"/>
+        <v>103</v>
+      </c>
+      <c r="C221" s="6"/>
+      <c r="D221" s="6"/>
+      <c r="E221" s="6"/>
+      <c r="F221" s="6"/>
+      <c r="G221" s="6"/>
+      <c r="H221" s="6"/>
+      <c r="I221" s="6"/>
+      <c r="J221" s="6"/>
+      <c r="K221" s="6"/>
+      <c r="L221" s="6"/>
+      <c r="M221" s="6"/>
+      <c r="N221" s="6"/>
+      <c r="O221" s="6"/>
+      <c r="P221" s="6"/>
+      <c r="Q221" s="6"/>
+      <c r="R221" s="6"/>
+      <c r="S221" s="6"/>
+      <c r="T221" s="6"/>
+      <c r="U221" s="6"/>
+      <c r="V221" s="6"/>
+      <c r="W221" s="6"/>
+      <c r="X221" s="6"/>
     </row>
     <row r="257" spans="2:17" ht="16.8" x14ac:dyDescent="0.3">
       <c r="B257" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="C257" s="4"/>
-      <c r="D257" s="4"/>
-      <c r="E257" s="4"/>
-      <c r="F257" s="4"/>
-      <c r="G257" s="4"/>
-      <c r="H257" s="4"/>
-      <c r="I257" s="4"/>
-      <c r="J257" s="4"/>
-      <c r="K257" s="4"/>
-      <c r="L257" s="4"/>
-      <c r="M257" s="4"/>
-      <c r="N257" s="4"/>
-      <c r="O257" s="4"/>
-      <c r="P257" s="4"/>
-      <c r="Q257" s="4"/>
+        <v>104</v>
+      </c>
+      <c r="C257" s="6"/>
+      <c r="D257" s="6"/>
+      <c r="E257" s="6"/>
+      <c r="F257" s="6"/>
+      <c r="G257" s="6"/>
+      <c r="H257" s="6"/>
+      <c r="I257" s="6"/>
+      <c r="J257" s="6"/>
+      <c r="K257" s="6"/>
+      <c r="L257" s="6"/>
+      <c r="M257" s="6"/>
+      <c r="N257" s="6"/>
+      <c r="O257" s="6"/>
+      <c r="P257" s="6"/>
+      <c r="Q257" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>